<commit_message>
régression flescher sur inflation et confiance
</commit_message>
<xml_diff>
--- a/data/data_inf.xlsx
+++ b/data/data_inf.xlsx
@@ -381,7 +381,7 @@
         <v>1996</v>
       </c>
       <c r="B2">
-        <v>0.002764793221279735</v>
+        <v>2.935579046620301</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -395,7 +395,7 @@
         <v>1997</v>
       </c>
       <c r="B3">
-        <v>0.001401061439130388</v>
+        <v>2.3408236004286</v>
       </c>
       <c r="C3">
         <v>1.6</v>
@@ -409,7 +409,7 @@
         <v>1998</v>
       </c>
       <c r="B4">
-        <v>0.001327235818096093</v>
+        <v>1.547044519209826</v>
       </c>
       <c r="C4">
         <v>1.1</v>
@@ -423,7 +423,7 @@
         <v>1999</v>
       </c>
       <c r="B5">
-        <v>0.002196796820900727</v>
+        <v>2.191477951890214</v>
       </c>
       <c r="C5">
         <v>1.1</v>
@@ -437,7 +437,7 @@
         <v>2000</v>
       </c>
       <c r="B6">
-        <v>0.002809258479985072</v>
+        <v>3.365998985841688</v>
       </c>
       <c r="C6">
         <v>2.1</v>
@@ -451,7 +451,7 @@
         <v>2001</v>
       </c>
       <c r="B7">
-        <v>0.001321670303165959</v>
+        <v>2.822433644618264</v>
       </c>
       <c r="C7">
         <v>2.3</v>
@@ -465,7 +465,7 @@
         <v>2002</v>
       </c>
       <c r="B8">
-        <v>0.002039142303531823</v>
+        <v>1.59492230330381</v>
       </c>
       <c r="C8">
         <v>2.3</v>
@@ -479,7 +479,7 @@
         <v>2003</v>
       </c>
       <c r="B9">
-        <v>0.001674018782389292</v>
+        <v>2.300187187577133</v>
       </c>
       <c r="C9">
         <v>2.1</v>
@@ -493,7 +493,7 @@
         <v>2004</v>
       </c>
       <c r="B10">
-        <v>0.002734596999368235</v>
+        <v>2.66615346051981</v>
       </c>
       <c r="C10">
         <v>2.2</v>
@@ -507,7 +507,7 @@
         <v>2005</v>
       </c>
       <c r="B11">
-        <v>0.002722924954980916</v>
+        <v>3.363331830947169</v>
       </c>
       <c r="C11">
         <v>2.2</v>
@@ -521,7 +521,7 @@
         <v>2006</v>
       </c>
       <c r="B12">
-        <v>0.002068807109105699</v>
+        <v>3.232509362248326</v>
       </c>
       <c r="C12">
         <v>2.2</v>
@@ -535,7 +535,7 @@
         <v>2007</v>
       </c>
       <c r="B13">
-        <v>0.003348206525929289</v>
+        <v>2.869311954703683</v>
       </c>
       <c r="C13">
         <v>2.1</v>
@@ -549,7 +549,7 @@
         <v>2008</v>
       </c>
       <c r="B14">
-        <v>-4.755017802572719E-05</v>
+        <v>3.825691321213462</v>
       </c>
       <c r="C14">
         <v>3.3</v>
@@ -563,7 +563,7 @@
         <v>2009</v>
       </c>
       <c r="B15">
-        <v>0.002307409948176967</v>
+        <v>-0.3073883011626958</v>
       </c>
       <c r="C15">
         <v>0.3</v>
@@ -577,7 +577,7 @@
         <v>2010</v>
       </c>
       <c r="B16">
-        <v>0.001187767786787087</v>
+        <v>1.640733389747095</v>
       </c>
       <c r="C16">
         <v>1.6</v>
@@ -591,7 +591,7 @@
         <v>2011</v>
       </c>
       <c r="B17">
-        <v>0.002509072184531059</v>
+        <v>3.138892794641766</v>
       </c>
       <c r="C17">
         <v>2.7</v>
@@ -605,7 +605,7 @@
         <v>2012</v>
       </c>
       <c r="B18">
-        <v>0.00144974039956031</v>
+        <v>2.076596904816102</v>
       </c>
       <c r="C18">
         <v>2.5</v>
@@ -619,7 +619,7 @@
         <v>2013</v>
       </c>
       <c r="B19">
-        <v>0.001248274020239947</v>
+        <v>1.467288583730721</v>
       </c>
       <c r="C19">
         <v>1.4</v>
@@ -633,7 +633,7 @@
         <v>2014</v>
       </c>
       <c r="B20">
-        <v>0.0005410610975057636</v>
+        <v>1.616629858562814</v>
       </c>
       <c r="C20">
         <v>0.4</v>
@@ -647,7 +647,7 @@
         <v>2015</v>
       </c>
       <c r="B21">
-        <v>0.0005270259897694992</v>
+        <v>0.1208393927813365</v>
       </c>
       <c r="C21">
         <v>0.2</v>
@@ -661,7 +661,7 @@
         <v>2016</v>
       </c>
       <c r="B22">
-        <v>0.001689071465350978</v>
+        <v>1.266680508170879</v>
       </c>
       <c r="C22">
         <v>0.2</v>
@@ -675,7 +675,7 @@
         <v>2017</v>
       </c>
       <c r="B23">
-        <v>0.001753203321375776</v>
+        <v>2.13267168250727</v>
       </c>
       <c r="C23">
         <v>1.5</v>
@@ -689,7 +689,7 @@
         <v>2018</v>
       </c>
       <c r="B24">
-        <v>0.001649982403116828</v>
+        <v>2.439754322318209</v>
       </c>
       <c r="C24">
         <v>1.8</v>
@@ -703,7 +703,7 @@
         <v>2019</v>
       </c>
       <c r="B25">
-        <v>0.001907907946896876</v>
+        <v>1.812632331534525</v>
       </c>
       <c r="C25">
         <v>1.2</v>
@@ -717,7 +717,7 @@
         <v>2020</v>
       </c>
       <c r="B26">
-        <v>0.001085477754010032</v>
+        <v>1.254878141114159</v>
       </c>
       <c r="C26">
         <v>0.3</v>
@@ -731,7 +731,7 @@
         <v>2021</v>
       </c>
       <c r="B27">
-        <v>0.005754769006530847</v>
+        <v>4.676516621102509</v>
       </c>
       <c r="C27">
         <v>2.6</v>
@@ -745,7 +745,7 @@
         <v>2022</v>
       </c>
       <c r="B28">
-        <v>0.005151713583089162</v>
+        <v>7.998425512331957</v>
       </c>
       <c r="C28">
         <v>8.4</v>
@@ -759,7 +759,7 @@
         <v>2023</v>
       </c>
       <c r="B29">
-        <v>0.002713840027534056</v>
+        <v>4.146104136642429</v>
       </c>
       <c r="C29">
         <v>5.5</v>
@@ -773,7 +773,7 @@
         <v>2024</v>
       </c>
       <c r="B30">
-        <v>0.002354866077240258</v>
+        <v>2.954307874795497</v>
       </c>
       <c r="C30">
         <v>2.4</v>

</xml_diff>